<commit_message>
Template: either ABC class or value (not both/partial), column notes; planner validates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/predlozak-popis-artikala.xlsx
+++ b/demo/predlozak-popis-artikala.xlsx
@@ -61,12 +61,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E55A00"/>
+        <fgColor rgb="005A6B8C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="005A6B8C"/>
+        <fgColor rgb="00E55A00"/>
       </patternFill>
     </fill>
   </fills>
@@ -175,6 +175,86 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Stanko Inventura</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>OBAVEZNO.
+Šifra artikla, jedinstvena za svaki redak (ista kao u vašem ERP-u/WMS-u). Duplikati se preskaču.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>NIJE OBAVEZNO, ali se preporučuje.
+Naziv artikla. Skladištar ga vidi na popisu za brojanje.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
+Ovaj stupac popunite ako već imate ABC klasu: upišite A, B ili C za SVE artikle. Tada stupac Vrijednost ostavite potpuno praznim.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
+Ovaj stupac popunite ako nemate ABC klasu: upišite godišnju vrijednost potrošnje (ili prometa) u EUR za SVE artikle. Aplikacija sama izračuna klase (A do 80 %, B do 95 %, ostalo C). Tada stupac ABC klasa ostavite potpuno praznim.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>NIJE OBAVEZNO.
+Bar kod (EAN) artikla; potreban samo za skeniranje kamerom. Bez njega se artikl na mobitelu bira s popisa. Stupac je tekstualni da se vodeće nule ne izgube.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Stanko Inventura</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>OBAVEZNO.
+Šifra artikla, jedinstvena za svaki redak (ista kao u vašem ERP-u/WMS-u). Duplikati se preskaču.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>NIJE OBAVEZNO, ali se preporučuje.
+Naziv artikla. Skladištar ga vidi na popisu za brojanje.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
+Ovaj stupac popunite ako već imate ABC klasu: upišite A, B ili C za SVE artikle. Tada stupac Vrijednost ostavite potpuno praznim.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
+Ovaj stupac popunite ako nemate ABC klasu: upišite godišnju vrijednost potrošnje (ili prometa) u EUR za SVE artikle. Aplikacija sama izračuna klase (A do 80 %, B do 95 %, ostalo C). Tada stupac ABC klasa ostavite potpuno praznim.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>NIJE OBAVEZNO.
+Bar kod (EAN) artikla; potreban samo za skeniranje kamerom. Bez njega se artikl na mobitelu bira s popisa. Stupac je tekstualni da se vodeće nule ne izgube.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -471,35 +551,35 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Šifra (obavezno)</t>
+          <t>Šifra</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Naziv</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>ABC klasa (ako je imate)</t>
+          <t>ABC klasa</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Vrijednost godišnje potrošnje, EUR (ako nemate klase)</t>
+          <t>Vrijednost godišnje potrošnje (EUR)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Bar kod (za skeniranje)</t>
+          <t>Bar kod</t>
         </is>
       </c>
     </row>
@@ -8505,11 +8585,12 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C20000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ABC klasa" error="Upišite A, B ili C (ili ostavite prazno)." type="list">
+    <dataValidation sqref="C2:C20000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ABC klasa" error="Upišite A, B ili C." type="list">
       <formula1>"A,B,C"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -8524,40 +8605,40 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Šifra (obavezno)</t>
+          <t>Šifra</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Naziv</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>ABC klasa (ako je imate)</t>
+          <t>ABC klasa</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Vrijednost godišnje potrošnje, EUR (ako nemate klase)</t>
+          <t>Vrijednost godišnje potrošnje (EUR)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Bar kod (za skeniranje)</t>
+          <t>Bar kod</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>Primjer: kod nekih artikala klasa je upisana, kod ostalih samo vrijednost. Aplikacija klasu izračuna samo tamo gdje je prazna.</t>
+          <t>Primjer s vrijednošću: stupac ABC klasa je prazan, a vrijednost je upisana za sve artikle. Ako imate klase, upišite ih za sve artikle, a stupac Vrijednost ostavite praznim.</t>
         </is>
       </c>
     </row>
@@ -8572,10 +8653,8 @@
           <t>Vijak M8 x 40</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="D2" t="n">
+        <v>125000</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
@@ -8634,10 +8713,8 @@
           <t>Ležaj 6204</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="D5" t="n">
+        <v>42000</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -8663,6 +8740,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -8672,7 +8750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -8688,63 +8766,70 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>1. Podatke upišite na listu „Artikli“ (od 2. retka). Zaglavlje ne brišite i ne premještajte.</t>
+          <t>1. Podatke upišite na list „Artikli“ od 2. retka. Zaglavlje ne brišite i ne premještajte. Opis svakog stupca i je li obavezan nalazi se u bilješci na zaglavlju (zadržite miš iznad ćelije).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>2. Šifra je jedina obavezna. Naziv preporučujemo jer ga skladištar vidi na popisu.</t>
+          <t>2. Šifra je obavezna. Naziv i bar kod nisu obavezni.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>3. ABC klasa: ako je već imate u sustavu, upišite A, B ili C.</t>
+          <t>3. Obavezno je popuniti JEDAN od dva stupca, za sve artikle:</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>4. Vrijednost: ako klase nemate, upišite godišnju vrijednost potrošnje (ili prometa) artikla u EUR. Aplikacija sama izračuna klase (Pareto: A do 80 % vrijednosti, B do 95 %, ostalo C).</t>
+          <t xml:space="preserve">      • ABC klasa: ako ABC klasu već imate. Upišite A, B ili C. Stupac Vrijednost ostavite praznim.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>5. Možete i miješati: gdje je klasa upisana, ostaje; gdje je prazna, računa se iz vrijednosti. Artikl bez klase i bez vrijednosti postaje C.</t>
+          <t xml:space="preserve">      • Vrijednost godišnje potrošnje (EUR): ako klasu nemate. Aplikacija je sama izračuna (Pareto: A do 80 %, B do 95 %, ostalo C). Stupac ABC klasa ostavite praznim.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>6. Bar kod (EAN) upišite ako želite skeniranje kamerom. Stupac je tekstualni da se vodeće nule ne izgube. Bez bar koda artikl se odabire s popisa.</t>
+          <t>4. Ne popunjavajte oba stupca i ne popunjavajte stupac samo za dio artikala: planer će javiti grešku.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>7. Datoteku učitajte u planer (ciklicka-inventura.html), generirajte raspored i preuzmite Excel s planom; njega učitajte u mobilnu aplikaciju.</t>
+          <t>5. Bar kod (EAN) upišite ako želite skeniranje kamerom; bez njega se artikl bira s popisa.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>8. Podaci ostaju na vašem računalu; ništa se ne šalje na internet.</t>
+          <t>6. Datoteku učitajte u planer, generirajte raspored i preuzmite Excel s planom; njega učitajte u mobilnu aplikaciju.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Ovaj list i list „Primjer“ ne utječu na učitavanje: planer čita samo prvi list („Artikli“).</t>
+          <t>7. Podaci ostaju na vašem računalu; ništa se ne šalje na internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Planer čita samo prvi list („Artikli“); listovi „Primjer“ i „Upute“ ne utječu na učitavanje.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planner: when both class and value are filled, use value
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/predlozak-popis-artikala.xlsx
+++ b/demo/predlozak-popis-artikala.xlsx
@@ -198,13 +198,13 @@
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
-Ovaj stupac popunite ako već imate ABC klasu: upišite A, B ili C za SVE artikle. Tada stupac Vrijednost ostavite potpuno praznim.</t>
+Ovaj stupac popunite ako već imate ABC klasu: upišite A, B ili C za SVE artikle. Tada stupac Vrijednost ostavite praznim. (Ako popunite oba stupca, planer koristi vrijednost.)</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
-Ovaj stupac popunite ako nemate ABC klasu: upišite godišnju vrijednost potrošnje (ili prometa) u EUR za SVE artikle. Aplikacija sama izračuna klase (A do 80 %, B do 95 %, ostalo C). Tada stupac ABC klasa ostavite potpuno praznim.</t>
+Ovaj stupac popunite ako nemate ABC klasu: upišite godišnju vrijednost potrošnje (ili prometa) u EUR za SVE artikle. Aplikacija sama izračuna klase (A do 80 %, B do 95 %, ostalo C). Tada stupac ABC klasa ostavite praznim.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -238,13 +238,13 @@
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
-Ovaj stupac popunite ako već imate ABC klasu: upišite A, B ili C za SVE artikle. Tada stupac Vrijednost ostavite potpuno praznim.</t>
+Ovaj stupac popunite ako već imate ABC klasu: upišite A, B ili C za SVE artikle. Tada stupac Vrijednost ostavite praznim. (Ako popunite oba stupca, planer koristi vrijednost.)</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>OBAVEZNO JE POPUNITI JEDAN OD DVA: ABC klasu ILI vrijednost.
-Ovaj stupac popunite ako nemate ABC klasu: upišite godišnju vrijednost potrošnje (ili prometa) u EUR za SVE artikle. Aplikacija sama izračuna klase (A do 80 %, B do 95 %, ostalo C). Tada stupac ABC klasa ostavite potpuno praznim.</t>
+Ovaj stupac popunite ako nemate ABC klasu: upišite godišnju vrijednost potrošnje (ili prometa) u EUR za SVE artikle. Aplikacija sama izračuna klase (A do 80 %, B do 95 %, ostalo C). Tada stupac ABC klasa ostavite praznim.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -8801,7 +8801,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>4. Ne popunjavajte oba stupca i ne popunjavajte stupac samo za dio artikala: planer će javiti grešku.</t>
+          <t>4. Ako popunite oba stupca, planer za izračun koristi vrijednost. Stupac popunjen samo za dio artikala planer odbija s greškom.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Guide and template: data format section
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/predlozak-popis-artikala.xlsx
+++ b/demo/predlozak-popis-artikala.xlsx
@@ -8750,7 +8750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -8806,28 +8806,77 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Format podataka (da se izbjegnu greške)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>• Šifra: jedinstvena za svaki redak; redak bez šifre i ponovljena šifra se preskaču.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>• ABC klasa: samo slovo A, B ili C, za sve artikle. Drugi znakovi odbacuju redak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>• Vrijednost: broj bez teksta, za sve artikle (npr. 12500 ili 12.500,50). Prazna ćelija nije dopuštena; ako artikl nema potrošnje, upišite 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>• Bar kod: samo znamenke (EAN-8, EAN-13), bez razmaka. Ćelije su već tekstualne; ako lijepite iz drugog izvora, zalijepite kao tekst da Excel ne obriše vodeće nule ili ne ispiše 3,86E+12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>• Zaglavlje je u prvom retku, a podaci odmah ispod. Bez praznih redaka, spojenih ćelija, međuzbrojeva i ukupnog retka na dnu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>• Podaci moraju biti na prvom listu. Preporučeni opseg: do oko 10.000 artikala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>5. Bar kod (EAN) upišite ako želite skeniranje kamerom; bez njega se artikl bira s popisa.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>6. Datoteku učitajte u planer, generirajte raspored i preuzmite Excel s planom; njega učitajte u mobilnu aplikaciju.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>7. Podaci ostaju na vašem računalu; ništa se ne šalje na internet.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Planer čita samo prvi list („Artikli“); listovi „Primjer“ i „Upute“ ne utječu na učitavanje.</t>
         </is>

</xml_diff>